<commit_message>
Cap nhat bao cao
</commit_message>
<xml_diff>
--- a/QLNS/FileExcels/SK_DanhSachCanBo_BVTV_01.xlsx
+++ b/QLNS/FileExcels/SK_DanhSachCanBo_BVTV_01.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9302"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="96" windowWidth="20112" windowHeight="8520"/>
@@ -12,12 +12,12 @@
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Danh sach can bo'!$1:$2</definedName>
   </definedNames>
-  <calcPr calcId="145621"/>
+  <calcPr calcId="144525"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="101">
   <si>
     <t>STT</t>
   </si>
@@ -115,9 +115,6 @@
     <t>(44)</t>
   </si>
   <si>
-    <t>Đơn vị/Phòng ban/Họ tên</t>
-  </si>
-  <si>
     <t>Mã CB</t>
   </si>
   <si>
@@ -314,6 +311,15 @@
   </si>
   <si>
     <t>HĐLĐ - Đến ngày</t>
+  </si>
+  <si>
+    <t>%TenDV_Child</t>
+  </si>
+  <si>
+    <t>Đơn vị/Phòng ban</t>
+  </si>
+  <si>
+    <t>Họ tên</t>
   </si>
 </sst>
 </file>
@@ -766,343 +772,351 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AH3"/>
+  <dimension ref="A1:AI3"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5.21875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="22.44140625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="7" style="1" customWidth="1"/>
-    <col min="4" max="4" width="9.77734375" style="6" customWidth="1"/>
-    <col min="5" max="5" width="5.33203125" style="1" customWidth="1"/>
-    <col min="6" max="6" width="13" style="1" customWidth="1"/>
-    <col min="7" max="7" width="9.77734375" style="1" customWidth="1"/>
-    <col min="8" max="8" width="14.88671875" style="1" customWidth="1"/>
-    <col min="9" max="12" width="20.77734375" style="1" customWidth="1"/>
-    <col min="13" max="13" width="5.33203125" style="1" customWidth="1"/>
-    <col min="14" max="14" width="6.5546875" style="1" customWidth="1"/>
-    <col min="15" max="15" width="8.88671875" style="1" customWidth="1"/>
-    <col min="16" max="16" width="12.33203125" style="1" customWidth="1"/>
-    <col min="17" max="17" width="14.109375" style="1" customWidth="1"/>
-    <col min="18" max="18" width="9.77734375" style="1" customWidth="1"/>
-    <col min="19" max="19" width="9.21875" style="1" customWidth="1"/>
-    <col min="20" max="20" width="13.6640625" style="1" customWidth="1"/>
-    <col min="21" max="22" width="9.5546875" style="1" customWidth="1"/>
-    <col min="23" max="23" width="10.33203125" style="1" customWidth="1"/>
-    <col min="24" max="24" width="14.88671875" style="1" customWidth="1"/>
-    <col min="25" max="25" width="6.33203125" style="1" customWidth="1"/>
-    <col min="26" max="26" width="6.21875" style="1" customWidth="1"/>
-    <col min="27" max="27" width="9.44140625" style="1" customWidth="1"/>
-    <col min="28" max="28" width="24.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="16.77734375" style="1" bestFit="1" customWidth="1"/>
-    <col min="30" max="33" width="9.77734375" style="1" customWidth="1"/>
-    <col min="34" max="34" width="23.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="35" max="16384" width="9.109375" style="1"/>
+    <col min="2" max="2" width="18.109375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="22.44140625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="7" style="1" customWidth="1"/>
+    <col min="5" max="5" width="9.77734375" style="6" customWidth="1"/>
+    <col min="6" max="6" width="5.33203125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="13" style="1" customWidth="1"/>
+    <col min="8" max="8" width="9.77734375" style="1" customWidth="1"/>
+    <col min="9" max="9" width="14.88671875" style="1" customWidth="1"/>
+    <col min="10" max="13" width="20.77734375" style="1" customWidth="1"/>
+    <col min="14" max="14" width="5.33203125" style="1" customWidth="1"/>
+    <col min="15" max="15" width="6.5546875" style="1" customWidth="1"/>
+    <col min="16" max="16" width="8.88671875" style="1" customWidth="1"/>
+    <col min="17" max="17" width="12.33203125" style="1" customWidth="1"/>
+    <col min="18" max="18" width="14.109375" style="1" customWidth="1"/>
+    <col min="19" max="19" width="9.77734375" style="1" customWidth="1"/>
+    <col min="20" max="20" width="9.21875" style="1" customWidth="1"/>
+    <col min="21" max="21" width="13.6640625" style="1" customWidth="1"/>
+    <col min="22" max="23" width="9.5546875" style="1" customWidth="1"/>
+    <col min="24" max="24" width="10.33203125" style="1" customWidth="1"/>
+    <col min="25" max="25" width="14.88671875" style="1" customWidth="1"/>
+    <col min="26" max="26" width="6.33203125" style="1" customWidth="1"/>
+    <col min="27" max="27" width="6.21875" style="1" customWidth="1"/>
+    <col min="28" max="28" width="9.44140625" style="1" customWidth="1"/>
+    <col min="29" max="29" width="24.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="16.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="31" max="34" width="9.77734375" style="1" customWidth="1"/>
+    <col min="35" max="35" width="23.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="36" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34" s="3" customFormat="1" ht="52.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:35" s="3" customFormat="1" ht="52.8" x14ac:dyDescent="0.3">
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="D1" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="E1" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="F1" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="G1" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="H1" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="G1" s="7" t="s">
+      <c r="I1" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="H1" s="7" t="s">
+      <c r="J1" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="I1" s="7" t="s">
+      <c r="K1" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="J1" s="7" t="s">
+      <c r="L1" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="K1" s="7" t="s">
+      <c r="M1" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="L1" s="7" t="s">
+      <c r="N1" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="M1" s="7" t="s">
+      <c r="O1" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="N1" s="7" t="s">
+      <c r="P1" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="Q1" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="O1" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="P1" s="8" t="s">
+      <c r="R1" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="Q1" s="8" t="s">
+      <c r="S1" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="R1" s="8" t="s">
+      <c r="T1" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="S1" s="8" t="s">
+      <c r="U1" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="T1" s="8" t="s">
+      <c r="V1" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="U1" s="8" t="s">
+      <c r="W1" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="X1" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="V1" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="W1" s="8" t="s">
+      <c r="Y1" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="X1" s="8" t="s">
+      <c r="Z1" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="Y1" s="8" t="s">
+      <c r="AA1" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="Z1" s="8" t="s">
+      <c r="AB1" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="AA1" s="8" t="s">
+      <c r="AC1" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="AB1" s="8" t="s">
+      <c r="AD1" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="AC1" s="8" t="s">
+      <c r="AE1" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="AD1" s="8" t="s">
+      <c r="AF1" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="AG1" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="AH1" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="AI1" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="AE1" s="8" t="s">
-        <v>97</v>
-      </c>
-      <c r="AF1" s="8" t="s">
-        <v>98</v>
-      </c>
-      <c r="AG1" s="8" t="s">
-        <v>96</v>
-      </c>
-      <c r="AH1" s="8" t="s">
-        <v>59</v>
-      </c>
     </row>
-    <row r="2" spans="1:34" s="2" customFormat="1" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:35" s="2" customFormat="1" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="5"/>
+      <c r="C2" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="D2" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="E2" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="F2" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="G2" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="G2" s="5" t="s">
+      <c r="H2" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="H2" s="5" t="s">
+      <c r="I2" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="I2" s="5" t="s">
+      <c r="J2" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="J2" s="5" t="s">
+      <c r="K2" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="K2" s="5" t="s">
+      <c r="L2" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="L2" s="5" t="s">
+      <c r="M2" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="M2" s="5" t="s">
+      <c r="N2" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="N2" s="5" t="s">
+      <c r="O2" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="O2" s="5" t="s">
+      <c r="P2" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="P2" s="5" t="s">
+      <c r="Q2" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="Q2" s="5" t="s">
+      <c r="R2" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="R2" s="5" t="s">
+      <c r="S2" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="S2" s="5" t="s">
+      <c r="T2" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="T2" s="5" t="s">
+      <c r="U2" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="U2" s="5" t="s">
+      <c r="V2" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="V2" s="5" t="s">
+      <c r="W2" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="W2" s="5" t="s">
+      <c r="X2" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="X2" s="5" t="s">
+      <c r="Y2" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="Y2" s="5" t="s">
+      <c r="Z2" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="Z2" s="5" t="s">
+      <c r="AA2" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="AA2" s="5" t="s">
+      <c r="AB2" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="AB2" s="5" t="s">
+      <c r="AC2" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="AC2" s="5" t="s">
+      <c r="AD2" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="AD2" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="AE2" s="5"/>
+      <c r="AE2" s="5" t="s">
+        <v>83</v>
+      </c>
       <c r="AF2" s="5"/>
       <c r="AG2" s="5"/>
-      <c r="AH2" s="5" t="s">
-        <v>92</v>
+      <c r="AH2" s="5"/>
+      <c r="AI2" s="5" t="s">
+        <v>91</v>
       </c>
     </row>
-    <row r="3" spans="1:34" s="3" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:35" s="3" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B3" s="9" t="s">
+      <c r="B3" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="C3" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="D3" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="E3" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="D3" s="10" t="s">
+      <c r="F3" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="E3" s="10" t="s">
+      <c r="G3" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="F3" s="10" t="s">
+      <c r="H3" s="10" t="s">
         <v>64</v>
       </c>
-      <c r="G3" s="10" t="s">
+      <c r="I3" s="11" t="s">
         <v>65</v>
       </c>
-      <c r="H3" s="11" t="s">
+      <c r="J3" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="I3" s="11" t="s">
+      <c r="K3" s="11" t="s">
         <v>67</v>
       </c>
-      <c r="J3" s="11" t="s">
+      <c r="L3" s="11" t="s">
         <v>68</v>
       </c>
-      <c r="K3" s="11" t="s">
+      <c r="M3" s="11" t="s">
         <v>69</v>
       </c>
-      <c r="L3" s="11" t="s">
+      <c r="N3" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="M3" s="10" t="s">
+      <c r="O3" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="N3" s="9" t="s">
+      <c r="P3" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="O3" s="11" t="s">
+      <c r="Q3" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="P3" s="10" t="s">
+      <c r="R3" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="Q3" s="9" t="s">
+      <c r="S3" s="10" t="s">
         <v>75</v>
       </c>
-      <c r="R3" s="10" t="s">
+      <c r="T3" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="S3" s="10" t="s">
+      <c r="U3" s="11" t="s">
         <v>77</v>
       </c>
-      <c r="T3" s="11" t="s">
+      <c r="V3" s="11" t="s">
         <v>78</v>
       </c>
-      <c r="U3" s="11" t="s">
+      <c r="W3" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="V3" s="11" t="s">
+      <c r="X3" s="11" t="s">
         <v>80</v>
       </c>
-      <c r="W3" s="11" t="s">
-        <v>81</v>
-      </c>
-      <c r="X3" s="11" t="s">
-        <v>83</v>
-      </c>
-      <c r="Y3" s="12" t="s">
+      <c r="Y3" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="Z3" s="12" t="s">
+        <v>84</v>
+      </c>
+      <c r="AA3" s="10" t="s">
         <v>85</v>
       </c>
-      <c r="Z3" s="10" t="s">
+      <c r="AB3" s="13" t="s">
         <v>86</v>
       </c>
-      <c r="AA3" s="13" t="s">
+      <c r="AC3" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="AB3" s="9" t="s">
+      <c r="AD3" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="AC3" s="9" t="s">
+      <c r="AE3" s="10" t="s">
         <v>89</v>
       </c>
-      <c r="AD3" s="10" t="s">
+      <c r="AF3" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="AG3" s="10" t="s">
+        <v>93</v>
+      </c>
+      <c r="AH3" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="AI3" s="11" t="s">
         <v>90</v>
-      </c>
-      <c r="AE3" s="10" t="s">
-        <v>93</v>
-      </c>
-      <c r="AF3" s="10" t="s">
-        <v>94</v>
-      </c>
-      <c r="AG3" s="11" t="s">
-        <v>95</v>
-      </c>
-      <c r="AH3" s="11" t="s">
-        <v>91</v>
       </c>
     </row>
   </sheetData>

</xml_diff>